<commit_message>
Respect Site Display tab so Bill 48 No hides the filter.
The converter only matched "Display Settings"; the live sheet tab is
"Site Display", so featured bills fell back to defaults that still
included Bill 48.
</commit_message>
<xml_diff>
--- a/Current Ontario MPPs & How They Vote..xlsx
+++ b/Current Ontario MPPs & How They Vote..xlsx
@@ -11,14 +11,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="8wtjvtIy+jYxcBMk+eUvWQQ8edLFPxK1cpyVj9xa6oA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="ug9ZCfUo/DnGAYg7wvZLeZQ/CAaP4zjSoqNJqMaAOdg="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3406" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3409" uniqueCount="1071">
   <si>
     <t>MPP Name</t>
   </si>
@@ -10006,11 +10006,7 @@
     <col customWidth="1" min="9" max="9" width="10.0"/>
     <col customWidth="1" min="10" max="10" width="20.0"/>
     <col customWidth="1" min="11" max="11" width="9.86"/>
-    <col customWidth="1" min="12" max="15" width="8.71"/>
-    <col customWidth="1" hidden="1" min="16" max="16" width="8.71"/>
-    <col customWidth="1" min="17" max="21" width="8.71"/>
-    <col customWidth="1" hidden="1" min="22" max="23" width="8.71"/>
-    <col customWidth="1" min="24" max="24" width="8.71"/>
+    <col customWidth="1" min="12" max="24" width="8.71"/>
     <col customWidth="1" min="25" max="25" width="9.86"/>
     <col customWidth="1" min="26" max="33" width="8.71"/>
     <col customWidth="1" min="34" max="34" width="13.57"/>
@@ -23274,7 +23270,7 @@
     </row>
     <row r="8">
       <c r="A8" s="60" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
       <c r="B8" s="62" t="s">
         <v>1069</v>
@@ -23285,7 +23281,7 @@
     </row>
     <row r="9">
       <c r="A9" s="60" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B9" s="62" t="s">
         <v>1069</v>
@@ -23296,7 +23292,7 @@
     </row>
     <row r="10">
       <c r="A10" s="60" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="B10" s="62" t="s">
         <v>1069</v>
@@ -23307,7 +23303,7 @@
     </row>
     <row r="11">
       <c r="A11" s="60" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="B11" s="62" t="s">
         <v>1069</v>
@@ -23318,7 +23314,7 @@
     </row>
     <row r="12">
       <c r="A12" s="60" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B12" s="62" t="s">
         <v>1069</v>
@@ -23329,7 +23325,7 @@
     </row>
     <row r="13">
       <c r="A13" s="60" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B13" s="62" t="s">
         <v>1069</v>
@@ -23340,12 +23336,23 @@
     </row>
     <row r="14">
       <c r="A14" s="60" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="B14" s="62" t="s">
         <v>1069</v>
       </c>
       <c r="C14" s="60" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="60" t="s">
+        <v>664</v>
+      </c>
+      <c r="B15" s="61" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C15" s="60" t="s">
         <v>1070</v>
       </c>
     </row>

</xml_diff>